<commit_message>
Shop: Kid nav, drop Unisex; image layout and CSV sync
- D2CStore: Kid category, remove Unisex; image borders/padding/clip tweaks
- csv-to-json: include products without local image files
- Update products.csv/xlsx, products.json, public/images

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="123">
   <si>
     <t>ID</t>
   </si>
@@ -255,6 +255,147 @@
   </si>
   <si>
     <t>LTGREYCLOUD</t>
+  </si>
+  <si>
+    <t>GUESS</t>
+  </si>
+  <si>
+    <t>NA-1</t>
+  </si>
+  <si>
+    <t>LADIES VEST</t>
+  </si>
+  <si>
+    <t>GREEN</t>
+  </si>
+  <si>
+    <t>Ladies, Vest, Outerwear</t>
+  </si>
+  <si>
+    <t>NA-2</t>
+  </si>
+  <si>
+    <t>LADIES DRAPE TOP</t>
+  </si>
+  <si>
+    <t>PINK</t>
+  </si>
+  <si>
+    <t>Ladies, Top, Drape</t>
+  </si>
+  <si>
+    <t>NA-3</t>
+  </si>
+  <si>
+    <t>LADIES RUFFLE-FLY NECK TANK TOP</t>
+  </si>
+  <si>
+    <t>PURPLE</t>
+  </si>
+  <si>
+    <t>Ladies, Tank Top, Ruffle</t>
+  </si>
+  <si>
+    <t>W01319-J44P0-B425-N</t>
+  </si>
+  <si>
+    <t>LADIES TOP</t>
+  </si>
+  <si>
+    <t>Ladies, Top</t>
+  </si>
+  <si>
+    <t>NA-4</t>
+  </si>
+  <si>
+    <t>BLUE</t>
+  </si>
+  <si>
+    <t>W31I45K21W0</t>
+  </si>
+  <si>
+    <t>GUESS KID</t>
+  </si>
+  <si>
+    <t>N01342-I3LI0</t>
+  </si>
+  <si>
+    <t>BOY POLO</t>
+  </si>
+  <si>
+    <t>NAVY</t>
+  </si>
+  <si>
+    <t>Kid, Boys, Polo</t>
+  </si>
+  <si>
+    <t>K01530-I3MQ0-B436-N</t>
+  </si>
+  <si>
+    <t>GIRL JACKET</t>
+  </si>
+  <si>
+    <t>Kid, Girls, Jacket</t>
+  </si>
+  <si>
+    <t>N01341-I3LI0</t>
+  </si>
+  <si>
+    <t>NA-5</t>
+  </si>
+  <si>
+    <t>GREY</t>
+  </si>
+  <si>
+    <t>J01351-I3QI0-001-N</t>
+  </si>
+  <si>
+    <t>GIRL TEE</t>
+  </si>
+  <si>
+    <t>WHITE</t>
+  </si>
+  <si>
+    <t>Kid, Girls, T-Shirt</t>
+  </si>
+  <si>
+    <t>J01355-I3QI0-B713-N</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>J01356-I3QI0-C457-N</t>
+  </si>
+  <si>
+    <t>GIRL SKIRT</t>
+  </si>
+  <si>
+    <t>Kid, Girls, Skirt, Bottoms</t>
+  </si>
+  <si>
+    <t>54_5</t>
+  </si>
+  <si>
+    <t>L01538I3MQ0-001-N</t>
+  </si>
+  <si>
+    <t>Kid, Girls, Jacket, Outerwear</t>
+  </si>
+  <si>
+    <t>NA-6</t>
+  </si>
+  <si>
+    <t>BOY JACKET</t>
+  </si>
+  <si>
+    <t>Kid, Boys, Jacket, Outerwear</t>
+  </si>
+  <si>
+    <t>L04532-I3MQ0-B446-N</t>
+  </si>
+  <si>
+    <t>L04534-I9AQ0-B446-N</t>
   </si>
 </sst>
 </file>
@@ -267,7 +408,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -300,6 +441,12 @@
       <name val="Arial"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.75"/>
+      <color rgb="FF0F1115"/>
+      <name val="Menlo"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
@@ -756,31 +903,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -789,119 +933,122 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -924,6 +1071,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1399,7 +1547,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:O1000"/>
+  <dimension ref="A1:O999"/>
   <sheetFormatPr defaultColWidth="12.6339285714286" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="7.25" style="1" customWidth="1"/>
@@ -1611,7 +1759,7 @@
         <v>13</v>
       </c>
       <c r="B7" s="4" t="str">
-        <f t="shared" ref="B7:B13" si="0">A7&amp;D7&amp;"_"&amp;F7</f>
+        <f t="shared" ref="B7:B17" si="0">A7&amp;D7&amp;"_"&amp;F7</f>
         <v>13AS151000_GREYMELANGE+OLDROSE</v>
       </c>
       <c r="C7" s="5" t="s">
@@ -1820,7 +1968,7 @@
         <v>46</v>
       </c>
       <c r="B14" s="4" t="str">
-        <f>A14&amp;D14&amp;"_"&amp;F14</f>
+        <f t="shared" si="0"/>
         <v>19_5MS14-1063_POWEREDROSESORBET</v>
       </c>
       <c r="C14" s="5" t="s">
@@ -1850,7 +1998,7 @@
         <v>20</v>
       </c>
       <c r="B15" s="4" t="str">
-        <f>A15&amp;D15&amp;"_"&amp;F15</f>
+        <f t="shared" si="0"/>
         <v>20MS14-1063_PINE</v>
       </c>
       <c r="C15" s="5" t="s">
@@ -1877,7 +2025,7 @@
         <v>21</v>
       </c>
       <c r="B16" s="4" t="str">
-        <f>A16&amp;D16&amp;"_"&amp;F16</f>
+        <f t="shared" si="0"/>
         <v>21MS14-1069_LIGHTGREY</v>
       </c>
       <c r="C16" s="5" t="s">
@@ -1904,7 +2052,7 @@
         <v>22</v>
       </c>
       <c r="B17" s="4" t="str">
-        <f>A17&amp;D17&amp;"_"&amp;F17</f>
+        <f t="shared" si="0"/>
         <v>22MS14-1069_POWDEREDROSESORBET</v>
       </c>
       <c r="C17" s="5" t="s">
@@ -2443,87 +2591,501 @@
       <c r="A37" s="1">
         <v>42</v>
       </c>
-      <c r="B37" s="4"/>
+      <c r="B37" s="4" t="str">
+        <f>A37&amp;D37&amp;"_"&amp;F37</f>
+        <v>42NA-1_GREEN</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="H37" s="1">
+        <v>1</v>
+      </c>
+      <c r="N37" s="8" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="38" customHeight="1" spans="1:14">
-      <c r="B38" s="4"/>
+      <c r="A38" s="1">
+        <v>43</v>
+      </c>
+      <c r="B38" s="4" t="str">
+        <f t="shared" ref="B37:B53" si="4">A38&amp;D38&amp;"_"&amp;F38</f>
+        <v>43NA-2_PINK</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H38" s="1">
+        <v>1</v>
+      </c>
+      <c r="N38" s="8" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="39" customHeight="1" spans="1:14">
-      <c r="B39" s="4"/>
+      <c r="A39" s="1">
+        <v>44</v>
+      </c>
+      <c r="B39" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>44NA-3_PURPLE</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="H39" s="1">
+        <v>1</v>
+      </c>
+      <c r="N39" s="8" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="40" customHeight="1" spans="1:14">
-      <c r="B40" s="4"/>
+      <c r="A40" s="1">
+        <v>45</v>
+      </c>
+      <c r="B40" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>45W01319-J44P0-B425-N_PINK</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H40" s="1">
+        <v>1</v>
+      </c>
+      <c r="N40" s="8" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="41" customHeight="1" spans="1:14">
-      <c r="B41" s="4"/>
+      <c r="A41" s="1">
+        <v>46</v>
+      </c>
+      <c r="B41" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>46NA-4_BLUE</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H41" s="1">
+        <v>1</v>
+      </c>
+      <c r="N41" s="8" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="42" customHeight="1" spans="1:14">
-      <c r="B42" s="4"/>
+      <c r="A42" s="1">
+        <v>47</v>
+      </c>
+      <c r="B42" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>47W31I45K21W0_BLUE</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H42" s="1">
+        <v>1</v>
+      </c>
+      <c r="N42" s="8" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="43" customHeight="1" spans="1:14">
-      <c r="B43" s="4"/>
+      <c r="A43" s="1">
+        <v>48</v>
+      </c>
+      <c r="B43" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>48N01342-I3LI0_NAVY</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="H43" s="1">
+        <v>1</v>
+      </c>
+      <c r="N43" s="8" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="44" customHeight="1" spans="1:14">
-      <c r="B44" s="4"/>
+      <c r="A44" s="1">
+        <v>49</v>
+      </c>
+      <c r="B44" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>49K01530-I3MQ0-B436-N_PINK</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H44" s="1">
+        <v>1</v>
+      </c>
+      <c r="N44" s="8" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="45" customHeight="1" spans="1:14">
-      <c r="B45" s="4"/>
+      <c r="A45" s="1">
+        <v>50</v>
+      </c>
+      <c r="B45" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>50N01341-I3LI0_BLUE</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I45" s="1">
+        <v>1</v>
+      </c>
+      <c r="N45" s="8" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="46" customHeight="1" spans="1:14">
-      <c r="B46" s="4"/>
+      <c r="A46" s="1">
+        <v>51</v>
+      </c>
+      <c r="B46" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>51NA-5_GREY</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="J46" s="1">
+        <v>1</v>
+      </c>
+      <c r="N46" s="8" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="47" customHeight="1" spans="1:14">
-      <c r="B47" s="4"/>
+      <c r="A47" s="1">
+        <v>52</v>
+      </c>
+      <c r="B47" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>52J01351-I3QI0-001-N_WHITE</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="H47" s="1">
+        <v>1</v>
+      </c>
+      <c r="N47" s="8" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="48" customHeight="1" spans="1:14">
-      <c r="B48" s="4"/>
-    </row>
-    <row r="49" customHeight="1" spans="2:2">
-      <c r="B49" s="4"/>
-    </row>
-    <row r="50" customHeight="1" spans="2:2">
-      <c r="B50" s="4"/>
-    </row>
-    <row r="51" customHeight="1" spans="2:2">
-      <c r="B51" s="4"/>
-    </row>
-    <row r="52" customHeight="1" spans="2:2">
-      <c r="B52" s="4"/>
-    </row>
-    <row r="53" customHeight="1" spans="2:2">
-      <c r="B53" s="4"/>
-    </row>
-    <row r="54" customHeight="1" spans="2:2">
+      <c r="A48" s="1">
+        <v>53</v>
+      </c>
+      <c r="B48" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>53J01355-I3QI0-B713-N_BLACK</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="I48" s="1">
+        <v>1</v>
+      </c>
+      <c r="J48" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="N48" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="49" customHeight="1" spans="1:14">
+      <c r="A49" s="1">
+        <v>54</v>
+      </c>
+      <c r="B49" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>54J01356-I3QI0-C457-N_PURPLE</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="H49" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="J49" s="1">
+        <v>1</v>
+      </c>
+      <c r="N49" s="8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="50" customHeight="1" spans="1:14">
+      <c r="A50" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B50" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>54_5L01538I3MQ0-001-N_WHITE</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="H50" s="1">
+        <v>1</v>
+      </c>
+      <c r="N50" s="8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="51" customHeight="1" spans="1:14">
+      <c r="A51" s="1">
+        <v>55</v>
+      </c>
+      <c r="B51" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>55NA-6_BLACK</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I51" s="1">
+        <v>1</v>
+      </c>
+      <c r="N51" s="8" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="52" customHeight="1" spans="1:14">
+      <c r="A52" s="1">
+        <v>56</v>
+      </c>
+      <c r="B52" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>56L04532-I3MQ0-B446-N_PURPLE</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="I52" s="1">
+        <v>1</v>
+      </c>
+      <c r="N52" s="8" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="53" customHeight="1" spans="1:14">
+      <c r="A53" s="1">
+        <v>57</v>
+      </c>
+      <c r="B53" s="4" t="str">
+        <f t="shared" si="4"/>
+        <v>57L04534-I9AQ0-B446-N_PURPLE</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="I53" s="1">
+        <v>1</v>
+      </c>
+      <c r="N53" s="8" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="54" customHeight="1" spans="1:14">
       <c r="B54" s="4"/>
     </row>
-    <row r="55" customHeight="1" spans="2:2">
+    <row r="55" customHeight="1" spans="1:14">
       <c r="B55" s="4"/>
     </row>
-    <row r="56" customHeight="1" spans="2:2">
+    <row r="56" customHeight="1" spans="1:14">
       <c r="B56" s="4"/>
     </row>
-    <row r="57" customHeight="1" spans="2:2">
+    <row r="57" customHeight="1" spans="1:14">
       <c r="B57" s="4"/>
     </row>
-    <row r="58" customHeight="1" spans="2:2">
+    <row r="58" customHeight="1" spans="1:14">
       <c r="B58" s="4"/>
     </row>
-    <row r="59" customHeight="1" spans="2:2">
+    <row r="59" customHeight="1" spans="1:14">
       <c r="B59" s="4"/>
     </row>
-    <row r="60" customHeight="1" spans="2:2">
+    <row r="60" customHeight="1" spans="1:14">
       <c r="B60" s="4"/>
     </row>
-    <row r="61" customHeight="1" spans="2:2">
+    <row r="61" customHeight="1" spans="1:14">
       <c r="B61" s="4"/>
     </row>
-    <row r="62" customHeight="1" spans="2:2">
+    <row r="62" customHeight="1" spans="1:14">
       <c r="B62" s="4"/>
     </row>
-    <row r="63" customHeight="1" spans="2:2">
+    <row r="63" customHeight="1" spans="1:14">
       <c r="B63" s="4"/>
     </row>
-    <row r="64" customHeight="1" spans="2:2">
+    <row r="64" customHeight="1" spans="1:14">
       <c r="B64" s="4"/>
     </row>
     <row r="65" customHeight="1" spans="2:2">
@@ -5330,9 +5892,6 @@
     </row>
     <row r="999" customHeight="1" spans="2:2">
       <c r="B999" s="4"/>
-    </row>
-    <row r="1000" customHeight="1" spans="2:2">
-      <c r="B1000" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sync products: CSV, products.json, and new images (59 items)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="140">
   <si>
     <t>ID</t>
   </si>
@@ -396,6 +396,57 @@
   </si>
   <si>
     <t>L04534-I9AQ0-B446-N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DESTINO </t>
+  </si>
+  <si>
+    <t>NA-7</t>
+  </si>
+  <si>
+    <t>Jogger - 100 modal</t>
+  </si>
+  <si>
+    <t>Bottoms</t>
+  </si>
+  <si>
+    <t>NA-8</t>
+  </si>
+  <si>
+    <t>shorts -100 modal</t>
+  </si>
+  <si>
+    <t>NA-9</t>
+  </si>
+  <si>
+    <t>v-neck top - 100 modal</t>
+  </si>
+  <si>
+    <t>Top</t>
+  </si>
+  <si>
+    <t>NA-10</t>
+  </si>
+  <si>
+    <t>full zip hoody - 100 modal</t>
+  </si>
+  <si>
+    <t>Top, Hoody</t>
+  </si>
+  <si>
+    <t>NA-11</t>
+  </si>
+  <si>
+    <t>tank top - two tone - 100 modal</t>
+  </si>
+  <si>
+    <t>NA-12</t>
+  </si>
+  <si>
+    <t>tank top - 100 modal</t>
+  </si>
+  <si>
+    <t>NA-13</t>
   </si>
 </sst>
 </file>
@@ -1554,7 +1605,7 @@
     <col min="2" max="2" width="29.3303571428571" style="1" customWidth="1"/>
     <col min="3" max="3" width="12.6339285714286" style="1"/>
     <col min="4" max="4" width="11.0714285714286" style="1" customWidth="1"/>
-    <col min="5" max="5" width="60.6696428571429" style="1" customWidth="1"/>
+    <col min="5" max="5" width="41.25" style="1" customWidth="1"/>
     <col min="6" max="6" width="26.5446428571429" style="1" customWidth="1"/>
     <col min="7" max="12" width="5.58035714285714" style="1" customWidth="1"/>
     <col min="13" max="13" width="6.58035714285714" style="1" customWidth="1"/>
@@ -2403,7 +2454,7 @@
         <v>35</v>
       </c>
       <c r="B30" s="4" t="str">
-        <f t="shared" ref="B30:B36" si="3">A30&amp;D30&amp;"_"&amp;F30</f>
+        <f t="shared" ref="B30:B37" si="3">A30&amp;D30&amp;"_"&amp;F30</f>
         <v>35MS14-1061_PINE</v>
       </c>
       <c r="C30" s="5" t="s">
@@ -2592,7 +2643,7 @@
         <v>42</v>
       </c>
       <c r="B37" s="4" t="str">
-        <f>A37&amp;D37&amp;"_"&amp;F37</f>
+        <f t="shared" si="3"/>
         <v>42NA-1_GREEN</v>
       </c>
       <c r="C37" s="1" t="s">
@@ -3056,25 +3107,160 @@
       </c>
     </row>
     <row r="54" customHeight="1" spans="1:14">
-      <c r="B54" s="4"/>
+      <c r="A54" s="1">
+        <v>1</v>
+      </c>
+      <c r="B54" s="4" t="str">
+        <f>A54&amp;D54</f>
+        <v>1NA-7</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="H54" s="1">
+        <v>1</v>
+      </c>
+      <c r="N54" s="2" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="55" customHeight="1" spans="1:14">
-      <c r="B55" s="4"/>
+      <c r="A55" s="1">
+        <v>2</v>
+      </c>
+      <c r="B55" s="4" t="str">
+        <f>A55&amp;D55</f>
+        <v>2NA-8</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="H55" s="1">
+        <v>1</v>
+      </c>
+      <c r="N55" s="2" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="56" customHeight="1" spans="1:14">
-      <c r="B56" s="4"/>
+      <c r="A56" s="1">
+        <v>3</v>
+      </c>
+      <c r="B56" s="4" t="str">
+        <f>A56&amp;D56</f>
+        <v>3NA-9</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="H56" s="1">
+        <v>1</v>
+      </c>
+      <c r="N56" s="2" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="57" customHeight="1" spans="1:14">
-      <c r="B57" s="4"/>
+      <c r="A57" s="1">
+        <v>4</v>
+      </c>
+      <c r="B57" s="4" t="str">
+        <f>A57&amp;D57</f>
+        <v>4NA-10</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="H57" s="1">
+        <v>1</v>
+      </c>
+      <c r="N57" s="2" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="58" customHeight="1" spans="1:14">
-      <c r="B58" s="4"/>
+      <c r="A58" s="1">
+        <v>5</v>
+      </c>
+      <c r="B58" s="4" t="str">
+        <f>A58&amp;D58</f>
+        <v>5NA-11</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="H58" s="1">
+        <v>1</v>
+      </c>
+      <c r="N58" s="2" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="59" customHeight="1" spans="1:14">
-      <c r="B59" s="4"/>
+      <c r="A59" s="1">
+        <v>6</v>
+      </c>
+      <c r="B59" s="4" t="str">
+        <f>A59&amp;D59</f>
+        <v>6NA-12</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="H59" s="1">
+        <v>1</v>
+      </c>
+      <c r="N59" s="2" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="60" customHeight="1" spans="1:14">
+      <c r="A60" s="1">
+        <v>7</v>
+      </c>
       <c r="B60" s="4"/>
+      <c r="C60" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="61" customHeight="1" spans="1:14">
       <c r="B61" s="4"/>

</xml_diff>